<commit_message>
fix: excel import format and structure.
</commit_message>
<xml_diff>
--- a/public/files/IQMY-Alpro Code Mapping Document 22July2025-ver1.1-NS.xlsx
+++ b/public/files/IQMY-Alpro Code Mapping Document 22July2025-ver1.1-NS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pathologyasia-my.sharepoint.com/personal/iqmy0959_pathologyasia_com/Documents/PROJECT - Integration/Alpro/Mapping/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\blood-stream-v1\public\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1216" documentId="8_{979185E3-AEED-4204-9A49-BEB87E4494B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E566046-781A-4DDD-BC0E-2237D8384C18}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB61A39D-7AEE-46E9-AD7B-99AB90CF0FD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28635" yWindow="-165" windowWidth="29130" windowHeight="15810" activeTab="3" xr2:uid="{90924F02-D7F6-4704-901E-FE125CE86CD4}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{90924F02-D7F6-4704-901E-FE125CE86CD4}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Panel Code" sheetId="2" r:id="rId1"/>
@@ -5769,7 +5769,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -5876,11 +5876,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -6707,7 +6703,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -6716,15 +6712,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7E33FC1-BD78-430F-8A03-094BFE5EB638}">
   <dimension ref="A1:D87"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="22.26953125" customWidth="1"/>
-    <col min="2" max="2" width="26.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.21875" customWidth="1"/>
+    <col min="2" max="2" width="26.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="35.5" customHeight="1">
+    <row r="1" spans="1:4" ht="35.549999999999997" customHeight="1">
       <c r="A1" s="6" t="s">
         <v>1785</v>
       </c>
@@ -7701,7 +7697,7 @@
         <v>1752</v>
       </c>
     </row>
-    <row r="83" spans="1:4" ht="20" customHeight="1">
+    <row r="83" spans="1:4" ht="19.95" customHeight="1">
       <c r="A83" t="s">
         <v>7</v>
       </c>
@@ -7726,7 +7722,7 @@
         <v>1787</v>
       </c>
     </row>
-    <row r="85" spans="1:4" ht="20" customHeight="1">
+    <row r="85" spans="1:4" ht="19.95" customHeight="1">
       <c r="A85" t="s">
         <v>24</v>
       </c>
@@ -7740,18 +7736,18 @@
         <v>1787</v>
       </c>
     </row>
-    <row r="86" spans="1:4" ht="20" customHeight="1"/>
-    <row r="87" spans="1:4" ht="20" customHeight="1"/>
+    <row r="86" spans="1:4" ht="19.95" customHeight="1"/>
+    <row r="87" spans="1:4" ht="19.95" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="14" type="noConversion"/>
-  <conditionalFormatting sqref="B1">
-    <cfRule type="duplicateValues" dxfId="2" priority="5"/>
+  <conditionalFormatting sqref="A1:A2">
+    <cfRule type="duplicateValues" dxfId="2" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:A1048576">
     <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A1:A2">
-    <cfRule type="duplicateValues" dxfId="0" priority="20"/>
+  <conditionalFormatting sqref="B1">
+    <cfRule type="duplicateValues" dxfId="0" priority="5"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -7763,16 +7759,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F4ED829-E96E-4333-996E-27CFBED2FDE1}">
   <dimension ref="A1:H251"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="23.81640625" customWidth="1"/>
-    <col min="2" max="2" width="21.26953125" customWidth="1"/>
-    <col min="3" max="3" width="7.90625" customWidth="1"/>
-    <col min="4" max="4" width="26.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.81640625" style="36" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.77734375" customWidth="1"/>
+    <col min="2" max="2" width="21.21875" customWidth="1"/>
+    <col min="3" max="3" width="7.88671875" customWidth="1"/>
+    <col min="4" max="4" width="26.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.77734375" style="36" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="37" customHeight="1">
+    <row r="1" spans="1:6" ht="37.049999999999997" customHeight="1">
       <c r="A1" s="34" t="s">
         <v>156</v>
       </c>
@@ -8540,20 +8536,20 @@
         <v>1748</v>
       </c>
     </row>
-    <row r="46" spans="1:5" s="42" customFormat="1">
-      <c r="A46" s="42" t="s">
+    <row r="46" spans="1:5">
+      <c r="A46" t="s">
         <v>131</v>
       </c>
-      <c r="B46" s="42" t="s">
+      <c r="B46" t="s">
         <v>1762</v>
       </c>
-      <c r="C46" s="42" t="s">
+      <c r="C46" t="s">
         <v>3</v>
       </c>
-      <c r="D46" s="42" t="s">
+      <c r="D46" t="s">
         <v>4</v>
       </c>
-      <c r="E46" s="44" t="s">
+      <c r="E46" s="36" t="s">
         <v>1741</v>
       </c>
     </row>
@@ -8897,20 +8893,20 @@
         <v>1748</v>
       </c>
     </row>
-    <row r="67" spans="1:5" s="42" customFormat="1">
-      <c r="A67" s="42" t="s">
+    <row r="67" spans="1:5">
+      <c r="A67" t="s">
         <v>111</v>
       </c>
-      <c r="B67" s="42" t="s">
+      <c r="B67" t="s">
         <v>1763</v>
       </c>
-      <c r="C67" s="42" t="s">
+      <c r="C67" t="s">
         <v>3</v>
       </c>
-      <c r="D67" s="42" t="s">
+      <c r="D67" t="s">
         <v>4</v>
       </c>
-      <c r="E67" s="44" t="s">
+      <c r="E67" s="36" t="s">
         <v>1741</v>
       </c>
     </row>
@@ -10342,7 +10338,7 @@
         <v>1748</v>
       </c>
     </row>
-    <row r="152" spans="1:5" ht="1" customHeight="1">
+    <row r="152" spans="1:5" ht="1.05" customHeight="1">
       <c r="A152" t="s">
         <v>52</v>
       </c>
@@ -12038,7 +12034,7 @@
       <c r="D251" s="40" t="s">
         <v>130</v>
       </c>
-      <c r="E251" s="43" t="s">
+      <c r="E251" s="42" t="s">
         <v>1748</v>
       </c>
       <c r="F251" s="40"/>
@@ -12059,14 +12055,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01D8B73B-281E-49E1-9ED7-16F79163D9A8}">
   <dimension ref="A1:E235"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="18.6328125" style="8" customWidth="1"/>
-    <col min="2" max="2" width="8.7265625" style="13"/>
-    <col min="3" max="3" width="21.36328125" style="13" customWidth="1"/>
-    <col min="4" max="4" width="32.81640625" style="16" customWidth="1"/>
-    <col min="5" max="5" width="48.54296875" style="14" customWidth="1"/>
-    <col min="6" max="16384" width="8.7265625" style="9"/>
+    <col min="1" max="1" width="18.6640625" style="8" customWidth="1"/>
+    <col min="2" max="2" width="8.77734375" style="13"/>
+    <col min="3" max="3" width="21.33203125" style="13" customWidth="1"/>
+    <col min="4" max="4" width="32.77734375" style="16" customWidth="1"/>
+    <col min="5" max="5" width="48.5546875" style="14" customWidth="1"/>
+    <col min="6" max="16384" width="8.77734375" style="9"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -12086,7 +12082,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="29">
+    <row r="2" spans="1:5" ht="28.8">
       <c r="A2" s="21" t="s">
         <v>407</v>
       </c>
@@ -12103,7 +12099,7 @@
         <v>1283</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="29">
+    <row r="3" spans="1:5" ht="28.8">
       <c r="A3" s="21" t="s">
         <v>407</v>
       </c>
@@ -12120,7 +12116,7 @@
         <v>1285</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="29">
+    <row r="4" spans="1:5" ht="28.8">
       <c r="A4" s="21" t="s">
         <v>407</v>
       </c>
@@ -12137,7 +12133,7 @@
         <v>1287</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="29">
+    <row r="5" spans="1:5" ht="28.8">
       <c r="A5" s="21" t="s">
         <v>407</v>
       </c>
@@ -12154,7 +12150,7 @@
         <v>1289</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="29">
+    <row r="6" spans="1:5" ht="28.8">
       <c r="A6" s="21" t="s">
         <v>407</v>
       </c>
@@ -12188,7 +12184,7 @@
         <v>1293</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="29">
+    <row r="8" spans="1:5">
       <c r="A8" s="21" t="s">
         <v>407</v>
       </c>
@@ -12205,7 +12201,7 @@
         <v>1295</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="29">
+    <row r="9" spans="1:5" ht="28.8">
       <c r="A9" s="21" t="s">
         <v>407</v>
       </c>
@@ -12222,7 +12218,7 @@
         <v>1297</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="29">
+    <row r="10" spans="1:5" ht="28.8">
       <c r="A10" s="21" t="s">
         <v>407</v>
       </c>
@@ -12239,7 +12235,7 @@
         <v>1299</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="29">
+    <row r="11" spans="1:5" ht="28.8">
       <c r="A11" s="21" t="s">
         <v>407</v>
       </c>
@@ -12256,7 +12252,7 @@
         <v>1301</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="29">
+    <row r="12" spans="1:5" ht="28.8">
       <c r="A12" s="21" t="s">
         <v>407</v>
       </c>
@@ -12273,7 +12269,7 @@
         <v>1303</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="29">
+    <row r="13" spans="1:5" ht="28.8">
       <c r="A13" s="21" t="s">
         <v>407</v>
       </c>
@@ -12290,7 +12286,7 @@
         <v>1305</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="29">
+    <row r="14" spans="1:5" ht="28.8">
       <c r="A14" s="21" t="s">
         <v>407</v>
       </c>
@@ -12307,7 +12303,7 @@
         <v>1307</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="29">
+    <row r="15" spans="1:5" ht="28.8">
       <c r="A15" s="21" t="s">
         <v>407</v>
       </c>
@@ -12324,7 +12320,7 @@
         <v>1309</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="29">
+    <row r="16" spans="1:5" ht="28.8">
       <c r="A16" s="21" t="s">
         <v>407</v>
       </c>
@@ -12341,7 +12337,7 @@
         <v>1311</v>
       </c>
     </row>
-    <row r="17" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="17" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A17" s="21" t="s">
         <v>407</v>
       </c>
@@ -12358,7 +12354,7 @@
         <v>1313</v>
       </c>
     </row>
-    <row r="18" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="18" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A18" s="21" t="s">
         <v>407</v>
       </c>
@@ -12375,7 +12371,7 @@
         <v>1315</v>
       </c>
     </row>
-    <row r="19" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="19" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A19" s="21" t="s">
         <v>407</v>
       </c>
@@ -12392,7 +12388,7 @@
         <v>1317</v>
       </c>
     </row>
-    <row r="20" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="20" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A20" s="21" t="s">
         <v>407</v>
       </c>
@@ -12426,7 +12422,7 @@
         <v>1321</v>
       </c>
     </row>
-    <row r="22" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="22" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A22" s="21" t="s">
         <v>407</v>
       </c>
@@ -12443,7 +12439,7 @@
         <v>1323</v>
       </c>
     </row>
-    <row r="23" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="23" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A23" s="21" t="s">
         <v>407</v>
       </c>
@@ -12460,7 +12456,7 @@
         <v>1325</v>
       </c>
     </row>
-    <row r="24" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="24" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A24" s="21" t="s">
         <v>407</v>
       </c>
@@ -12477,7 +12473,7 @@
         <v>1327</v>
       </c>
     </row>
-    <row r="25" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="25" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A25" s="21" t="s">
         <v>407</v>
       </c>
@@ -12494,7 +12490,7 @@
         <v>1329</v>
       </c>
     </row>
-    <row r="26" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="26" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A26" s="21" t="s">
         <v>407</v>
       </c>
@@ -12511,7 +12507,7 @@
         <v>1331</v>
       </c>
     </row>
-    <row r="27" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="27" spans="1:5" s="12" customFormat="1">
       <c r="A27" s="21" t="s">
         <v>407</v>
       </c>
@@ -12545,7 +12541,7 @@
         <v>1335</v>
       </c>
     </row>
-    <row r="29" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="29" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A29" s="21" t="s">
         <v>407</v>
       </c>
@@ -12562,7 +12558,7 @@
         <v>1337</v>
       </c>
     </row>
-    <row r="30" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="30" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A30" s="21" t="s">
         <v>407</v>
       </c>
@@ -12579,7 +12575,7 @@
         <v>1339</v>
       </c>
     </row>
-    <row r="31" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="31" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A31" s="21" t="s">
         <v>407</v>
       </c>
@@ -12596,7 +12592,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="32" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="32" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A32" s="21" t="s">
         <v>407</v>
       </c>
@@ -12613,7 +12609,7 @@
         <v>1343</v>
       </c>
     </row>
-    <row r="33" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="33" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A33" s="21" t="s">
         <v>407</v>
       </c>
@@ -12630,7 +12626,7 @@
         <v>1345</v>
       </c>
     </row>
-    <row r="34" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="34" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A34" s="21" t="s">
         <v>407</v>
       </c>
@@ -12647,7 +12643,7 @@
         <v>1347</v>
       </c>
     </row>
-    <row r="35" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="35" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A35" s="21" t="s">
         <v>407</v>
       </c>
@@ -12681,7 +12677,7 @@
         <v>1351</v>
       </c>
     </row>
-    <row r="37" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="37" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A37" s="21" t="s">
         <v>407</v>
       </c>
@@ -12698,7 +12694,7 @@
         <v>1353</v>
       </c>
     </row>
-    <row r="38" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="38" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A38" s="21" t="s">
         <v>407</v>
       </c>
@@ -12715,7 +12711,7 @@
         <v>1355</v>
       </c>
     </row>
-    <row r="39" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="39" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A39" s="21" t="s">
         <v>407</v>
       </c>
@@ -12732,7 +12728,7 @@
         <v>1357</v>
       </c>
     </row>
-    <row r="40" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="40" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A40" s="21" t="s">
         <v>407</v>
       </c>
@@ -12749,7 +12745,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="41" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="41" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A41" s="21" t="s">
         <v>407</v>
       </c>
@@ -12766,7 +12762,7 @@
         <v>1361</v>
       </c>
     </row>
-    <row r="42" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="42" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A42" s="21" t="s">
         <v>407</v>
       </c>
@@ -12783,7 +12779,7 @@
         <v>1363</v>
       </c>
     </row>
-    <row r="43" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="43" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A43" s="21" t="s">
         <v>407</v>
       </c>
@@ -12800,7 +12796,7 @@
         <v>1365</v>
       </c>
     </row>
-    <row r="44" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="44" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A44" s="21" t="s">
         <v>407</v>
       </c>
@@ -12817,7 +12813,7 @@
         <v>1367</v>
       </c>
     </row>
-    <row r="45" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="45" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A45" s="21" t="s">
         <v>407</v>
       </c>
@@ -12851,7 +12847,7 @@
         <v>1371</v>
       </c>
     </row>
-    <row r="47" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="47" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A47" s="21" t="s">
         <v>407</v>
       </c>
@@ -12868,7 +12864,7 @@
         <v>1373</v>
       </c>
     </row>
-    <row r="48" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="48" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A48" s="21" t="s">
         <v>407</v>
       </c>
@@ -12885,7 +12881,7 @@
         <v>1375</v>
       </c>
     </row>
-    <row r="49" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="49" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A49" s="21" t="s">
         <v>407</v>
       </c>
@@ -12902,7 +12898,7 @@
         <v>1377</v>
       </c>
     </row>
-    <row r="50" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="50" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A50" s="21" t="s">
         <v>407</v>
       </c>
@@ -12919,7 +12915,7 @@
         <v>1379</v>
       </c>
     </row>
-    <row r="51" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="51" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A51" s="21" t="s">
         <v>407</v>
       </c>
@@ -12936,7 +12932,7 @@
         <v>1381</v>
       </c>
     </row>
-    <row r="52" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="52" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A52" s="21" t="s">
         <v>407</v>
       </c>
@@ -12953,7 +12949,7 @@
         <v>1383</v>
       </c>
     </row>
-    <row r="53" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="53" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A53" s="21" t="s">
         <v>407</v>
       </c>
@@ -12970,7 +12966,7 @@
         <v>1385</v>
       </c>
     </row>
-    <row r="54" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="54" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A54" s="21" t="s">
         <v>407</v>
       </c>
@@ -12987,7 +12983,7 @@
         <v>1387</v>
       </c>
     </row>
-    <row r="55" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="55" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A55" s="21" t="s">
         <v>407</v>
       </c>
@@ -13004,7 +13000,7 @@
         <v>1389</v>
       </c>
     </row>
-    <row r="56" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="56" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A56" s="21" t="s">
         <v>407</v>
       </c>
@@ -13021,7 +13017,7 @@
         <v>1391</v>
       </c>
     </row>
-    <row r="57" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="57" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A57" s="21" t="s">
         <v>407</v>
       </c>
@@ -13038,7 +13034,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="58" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="58" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A58" s="21" t="s">
         <v>407</v>
       </c>
@@ -13055,7 +13051,7 @@
         <v>1395</v>
       </c>
     </row>
-    <row r="59" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="59" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A59" s="21" t="s">
         <v>407</v>
       </c>
@@ -13072,7 +13068,7 @@
         <v>1397</v>
       </c>
     </row>
-    <row r="60" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="60" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A60" s="21" t="s">
         <v>407</v>
       </c>
@@ -13089,7 +13085,7 @@
         <v>1399</v>
       </c>
     </row>
-    <row r="61" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="61" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A61" s="21" t="s">
         <v>407</v>
       </c>
@@ -13106,7 +13102,7 @@
         <v>1401</v>
       </c>
     </row>
-    <row r="62" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="62" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A62" s="21" t="s">
         <v>407</v>
       </c>
@@ -13123,7 +13119,7 @@
         <v>1403</v>
       </c>
     </row>
-    <row r="63" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="63" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A63" s="21" t="s">
         <v>407</v>
       </c>
@@ -13140,7 +13136,7 @@
         <v>1405</v>
       </c>
     </row>
-    <row r="64" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="64" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A64" s="21" t="s">
         <v>407</v>
       </c>
@@ -13157,7 +13153,7 @@
         <v>1407</v>
       </c>
     </row>
-    <row r="65" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="65" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A65" s="21" t="s">
         <v>407</v>
       </c>
@@ -13174,7 +13170,7 @@
         <v>1409</v>
       </c>
     </row>
-    <row r="66" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="66" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A66" s="21" t="s">
         <v>407</v>
       </c>
@@ -13191,7 +13187,7 @@
         <v>1411</v>
       </c>
     </row>
-    <row r="67" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="67" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A67" s="21" t="s">
         <v>407</v>
       </c>
@@ -13208,7 +13204,7 @@
         <v>1413</v>
       </c>
     </row>
-    <row r="68" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="68" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A68" s="21" t="s">
         <v>407</v>
       </c>
@@ -13225,7 +13221,7 @@
         <v>1415</v>
       </c>
     </row>
-    <row r="69" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="69" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A69" s="21" t="s">
         <v>407</v>
       </c>
@@ -13242,7 +13238,7 @@
         <v>1417</v>
       </c>
     </row>
-    <row r="70" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="70" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A70" s="21" t="s">
         <v>407</v>
       </c>
@@ -13259,7 +13255,7 @@
         <v>1419</v>
       </c>
     </row>
-    <row r="71" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="71" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A71" s="21" t="s">
         <v>407</v>
       </c>
@@ -13276,7 +13272,7 @@
         <v>1421</v>
       </c>
     </row>
-    <row r="72" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="72" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A72" s="21" t="s">
         <v>407</v>
       </c>
@@ -13293,7 +13289,7 @@
         <v>1423</v>
       </c>
     </row>
-    <row r="73" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="73" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A73" s="21" t="s">
         <v>407</v>
       </c>
@@ -13310,7 +13306,7 @@
         <v>1425</v>
       </c>
     </row>
-    <row r="74" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="74" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A74" s="21" t="s">
         <v>407</v>
       </c>
@@ -13327,7 +13323,7 @@
         <v>1427</v>
       </c>
     </row>
-    <row r="75" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="75" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A75" s="21" t="s">
         <v>407</v>
       </c>
@@ -13344,7 +13340,7 @@
         <v>1429</v>
       </c>
     </row>
-    <row r="76" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="76" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A76" s="21" t="s">
         <v>407</v>
       </c>
@@ -13361,7 +13357,7 @@
         <v>1431</v>
       </c>
     </row>
-    <row r="77" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="77" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A77" s="21" t="s">
         <v>407</v>
       </c>
@@ -13378,7 +13374,7 @@
         <v>1433</v>
       </c>
     </row>
-    <row r="78" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="78" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A78" s="21" t="s">
         <v>407</v>
       </c>
@@ -13446,7 +13442,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="82" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="82" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A82" s="21" t="s">
         <v>407</v>
       </c>
@@ -13463,7 +13459,7 @@
         <v>1443</v>
       </c>
     </row>
-    <row r="83" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="83" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A83" s="21" t="s">
         <v>407</v>
       </c>
@@ -13480,7 +13476,7 @@
         <v>1445</v>
       </c>
     </row>
-    <row r="84" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="84" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A84" s="21" t="s">
         <v>407</v>
       </c>
@@ -13514,7 +13510,7 @@
         <v>1449</v>
       </c>
     </row>
-    <row r="86" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="86" spans="1:5" s="12" customFormat="1">
       <c r="A86" s="21" t="s">
         <v>407</v>
       </c>
@@ -13531,7 +13527,7 @@
         <v>1451</v>
       </c>
     </row>
-    <row r="87" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="87" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A87" s="21" t="s">
         <v>407</v>
       </c>
@@ -13548,7 +13544,7 @@
         <v>1453</v>
       </c>
     </row>
-    <row r="88" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="88" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A88" s="21" t="s">
         <v>407</v>
       </c>
@@ -13565,7 +13561,7 @@
         <v>1455</v>
       </c>
     </row>
-    <row r="89" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="89" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A89" s="21" t="s">
         <v>407</v>
       </c>
@@ -13582,7 +13578,7 @@
         <v>1457</v>
       </c>
     </row>
-    <row r="90" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="90" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A90" s="21" t="s">
         <v>407</v>
       </c>
@@ -13599,7 +13595,7 @@
         <v>1459</v>
       </c>
     </row>
-    <row r="91" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="91" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A91" s="21" t="s">
         <v>407</v>
       </c>
@@ -13633,7 +13629,7 @@
         <v>1463</v>
       </c>
     </row>
-    <row r="93" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="93" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A93" s="21" t="s">
         <v>407</v>
       </c>
@@ -13667,7 +13663,7 @@
         <v>1467</v>
       </c>
     </row>
-    <row r="95" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="95" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A95" s="21" t="s">
         <v>407</v>
       </c>
@@ -13684,7 +13680,7 @@
         <v>1469</v>
       </c>
     </row>
-    <row r="96" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="96" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A96" s="21" t="s">
         <v>407</v>
       </c>
@@ -13701,7 +13697,7 @@
         <v>1471</v>
       </c>
     </row>
-    <row r="97" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="97" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A97" s="21" t="s">
         <v>407</v>
       </c>
@@ -13718,7 +13714,7 @@
         <v>1473</v>
       </c>
     </row>
-    <row r="98" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="98" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A98" s="21" t="s">
         <v>407</v>
       </c>
@@ -13735,7 +13731,7 @@
         <v>1475</v>
       </c>
     </row>
-    <row r="99" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="99" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A99" s="21" t="s">
         <v>407</v>
       </c>
@@ -13752,7 +13748,7 @@
         <v>1477</v>
       </c>
     </row>
-    <row r="100" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="100" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A100" s="21" t="s">
         <v>407</v>
       </c>
@@ -13786,7 +13782,7 @@
         <v>1481</v>
       </c>
     </row>
-    <row r="102" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="102" spans="1:5" s="12" customFormat="1">
       <c r="A102" s="21" t="s">
         <v>407</v>
       </c>
@@ -13820,7 +13816,7 @@
         <v>1485</v>
       </c>
     </row>
-    <row r="104" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="104" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A104" s="21" t="s">
         <v>407</v>
       </c>
@@ -13837,7 +13833,7 @@
         <v>1487</v>
       </c>
     </row>
-    <row r="105" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="105" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A105" s="21" t="s">
         <v>407</v>
       </c>
@@ -13854,7 +13850,7 @@
         <v>1489</v>
       </c>
     </row>
-    <row r="106" spans="1:5" s="12" customFormat="1" ht="43.5">
+    <row r="106" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A106" s="21" t="s">
         <v>407</v>
       </c>
@@ -13871,7 +13867,7 @@
         <v>1491</v>
       </c>
     </row>
-    <row r="107" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="107" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A107" s="21" t="s">
         <v>407</v>
       </c>
@@ -13888,7 +13884,7 @@
         <v>1493</v>
       </c>
     </row>
-    <row r="108" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="108" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A108" s="21" t="s">
         <v>407</v>
       </c>
@@ -13905,7 +13901,7 @@
         <v>1495</v>
       </c>
     </row>
-    <row r="109" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="109" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A109" s="21" t="s">
         <v>407</v>
       </c>
@@ -13922,7 +13918,7 @@
         <v>1497</v>
       </c>
     </row>
-    <row r="110" spans="1:5" s="12" customFormat="1" ht="43.5">
+    <row r="110" spans="1:5" s="12" customFormat="1" ht="43.2">
       <c r="A110" s="21" t="s">
         <v>407</v>
       </c>
@@ -13939,7 +13935,7 @@
         <v>1499</v>
       </c>
     </row>
-    <row r="111" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="111" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A111" s="21" t="s">
         <v>407</v>
       </c>
@@ -13956,7 +13952,7 @@
         <v>1501</v>
       </c>
     </row>
-    <row r="112" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="112" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A112" s="21" t="s">
         <v>407</v>
       </c>
@@ -13973,7 +13969,7 @@
         <v>1503</v>
       </c>
     </row>
-    <row r="113" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="113" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A113" s="21" t="s">
         <v>407</v>
       </c>
@@ -13990,7 +13986,7 @@
         <v>1505</v>
       </c>
     </row>
-    <row r="114" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="114" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A114" s="21" t="s">
         <v>407</v>
       </c>
@@ -14007,7 +14003,7 @@
         <v>1507</v>
       </c>
     </row>
-    <row r="115" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="115" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A115" s="21" t="s">
         <v>407</v>
       </c>
@@ -14024,7 +14020,7 @@
         <v>1509</v>
       </c>
     </row>
-    <row r="116" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="116" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A116" s="21" t="s">
         <v>407</v>
       </c>
@@ -14041,7 +14037,7 @@
         <v>1511</v>
       </c>
     </row>
-    <row r="117" spans="1:5" s="12" customFormat="1" ht="43.5">
+    <row r="117" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A117" s="21" t="s">
         <v>407</v>
       </c>
@@ -14058,7 +14054,7 @@
         <v>1513</v>
       </c>
     </row>
-    <row r="118" spans="1:5" s="12" customFormat="1" ht="43.5">
+    <row r="118" spans="1:5" s="12" customFormat="1" ht="43.2">
       <c r="A118" s="21" t="s">
         <v>407</v>
       </c>
@@ -14075,7 +14071,7 @@
         <v>1515</v>
       </c>
     </row>
-    <row r="119" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="119" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A119" s="21" t="s">
         <v>407</v>
       </c>
@@ -14092,7 +14088,7 @@
         <v>1517</v>
       </c>
     </row>
-    <row r="120" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="120" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A120" s="21" t="s">
         <v>407</v>
       </c>
@@ -14109,7 +14105,7 @@
         <v>1519</v>
       </c>
     </row>
-    <row r="121" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="121" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A121" s="21" t="s">
         <v>407</v>
       </c>
@@ -14126,7 +14122,7 @@
         <v>1521</v>
       </c>
     </row>
-    <row r="122" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="122" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A122" s="21" t="s">
         <v>407</v>
       </c>
@@ -14143,7 +14139,7 @@
         <v>1523</v>
       </c>
     </row>
-    <row r="123" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="123" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A123" s="21" t="s">
         <v>407</v>
       </c>
@@ -14160,7 +14156,7 @@
         <v>1525</v>
       </c>
     </row>
-    <row r="124" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="124" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A124" s="21" t="s">
         <v>407</v>
       </c>
@@ -14228,7 +14224,7 @@
         <v>1533</v>
       </c>
     </row>
-    <row r="128" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="128" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A128" s="21" t="s">
         <v>407</v>
       </c>
@@ -14245,7 +14241,7 @@
         <v>1535</v>
       </c>
     </row>
-    <row r="129" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="129" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A129" s="21" t="s">
         <v>407</v>
       </c>
@@ -14262,7 +14258,7 @@
         <v>1537</v>
       </c>
     </row>
-    <row r="130" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="130" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A130" s="21" t="s">
         <v>407</v>
       </c>
@@ -14279,7 +14275,7 @@
         <v>1539</v>
       </c>
     </row>
-    <row r="131" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="131" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A131" s="21" t="s">
         <v>407</v>
       </c>
@@ -14296,7 +14292,7 @@
         <v>1541</v>
       </c>
     </row>
-    <row r="132" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="132" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A132" s="21" t="s">
         <v>407</v>
       </c>
@@ -14330,7 +14326,7 @@
         <v>1545</v>
       </c>
     </row>
-    <row r="134" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="134" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A134" s="21" t="s">
         <v>407</v>
       </c>
@@ -14347,7 +14343,7 @@
         <v>1547</v>
       </c>
     </row>
-    <row r="135" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="135" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A135" s="21" t="s">
         <v>407</v>
       </c>
@@ -14364,7 +14360,7 @@
         <v>1549</v>
       </c>
     </row>
-    <row r="136" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="136" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A136" s="21" t="s">
         <v>407</v>
       </c>
@@ -14398,7 +14394,7 @@
         <v>1553</v>
       </c>
     </row>
-    <row r="138" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="138" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A138" s="21" t="s">
         <v>407</v>
       </c>
@@ -14415,7 +14411,7 @@
         <v>1555</v>
       </c>
     </row>
-    <row r="139" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="139" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A139" s="21" t="s">
         <v>407</v>
       </c>
@@ -14432,7 +14428,7 @@
         <v>1557</v>
       </c>
     </row>
-    <row r="140" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="140" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A140" s="21" t="s">
         <v>407</v>
       </c>
@@ -14449,7 +14445,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="141" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="141" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A141" s="21" t="s">
         <v>407</v>
       </c>
@@ -14466,7 +14462,7 @@
         <v>1561</v>
       </c>
     </row>
-    <row r="142" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="142" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A142" s="21" t="s">
         <v>407</v>
       </c>
@@ -14483,7 +14479,7 @@
         <v>1563</v>
       </c>
     </row>
-    <row r="143" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="143" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A143" s="21" t="s">
         <v>407</v>
       </c>
@@ -14500,7 +14496,7 @@
         <v>1565</v>
       </c>
     </row>
-    <row r="144" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="144" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A144" s="21" t="s">
         <v>407</v>
       </c>
@@ -14517,7 +14513,7 @@
         <v>1567</v>
       </c>
     </row>
-    <row r="145" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="145" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A145" s="21" t="s">
         <v>407</v>
       </c>
@@ -14551,7 +14547,7 @@
         <v>1571</v>
       </c>
     </row>
-    <row r="147" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="147" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A147" s="21" t="s">
         <v>407</v>
       </c>
@@ -14568,7 +14564,7 @@
         <v>1573</v>
       </c>
     </row>
-    <row r="148" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="148" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A148" s="21" t="s">
         <v>407</v>
       </c>
@@ -14585,7 +14581,7 @@
         <v>1575</v>
       </c>
     </row>
-    <row r="149" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="149" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A149" s="21" t="s">
         <v>407</v>
       </c>
@@ -14602,7 +14598,7 @@
         <v>1577</v>
       </c>
     </row>
-    <row r="150" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="150" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A150" s="21" t="s">
         <v>407</v>
       </c>
@@ -14619,7 +14615,7 @@
         <v>1579</v>
       </c>
     </row>
-    <row r="151" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="151" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A151" s="21" t="s">
         <v>407</v>
       </c>
@@ -14636,7 +14632,7 @@
         <v>1581</v>
       </c>
     </row>
-    <row r="152" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="152" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A152" s="21" t="s">
         <v>407</v>
       </c>
@@ -14653,7 +14649,7 @@
         <v>1583</v>
       </c>
     </row>
-    <row r="153" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="153" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A153" s="21" t="s">
         <v>407</v>
       </c>
@@ -14687,7 +14683,7 @@
         <v>1587</v>
       </c>
     </row>
-    <row r="155" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="155" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A155" s="21" t="s">
         <v>407</v>
       </c>
@@ -14704,7 +14700,7 @@
         <v>1589</v>
       </c>
     </row>
-    <row r="156" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="156" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A156" s="21" t="s">
         <v>407</v>
       </c>
@@ -14721,7 +14717,7 @@
         <v>1591</v>
       </c>
     </row>
-    <row r="157" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="157" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A157" s="21" t="s">
         <v>407</v>
       </c>
@@ -14738,7 +14734,7 @@
         <v>1593</v>
       </c>
     </row>
-    <row r="158" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="158" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A158" s="21" t="s">
         <v>407</v>
       </c>
@@ -14755,7 +14751,7 @@
         <v>1595</v>
       </c>
     </row>
-    <row r="159" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="159" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A159" s="21" t="s">
         <v>407</v>
       </c>
@@ -14772,7 +14768,7 @@
         <v>1597</v>
       </c>
     </row>
-    <row r="160" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="160" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A160" s="21" t="s">
         <v>407</v>
       </c>
@@ -14789,7 +14785,7 @@
         <v>1599</v>
       </c>
     </row>
-    <row r="161" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="161" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A161" s="21" t="s">
         <v>407</v>
       </c>
@@ -14806,7 +14802,7 @@
         <v>1601</v>
       </c>
     </row>
-    <row r="162" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="162" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A162" s="21" t="s">
         <v>407</v>
       </c>
@@ -14823,7 +14819,7 @@
         <v>1603</v>
       </c>
     </row>
-    <row r="163" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="163" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A163" s="21" t="s">
         <v>407</v>
       </c>
@@ -14840,7 +14836,7 @@
         <v>1605</v>
       </c>
     </row>
-    <row r="164" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="164" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A164" s="21" t="s">
         <v>407</v>
       </c>
@@ -14857,7 +14853,7 @@
         <v>1607</v>
       </c>
     </row>
-    <row r="165" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="165" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A165" s="21" t="s">
         <v>407</v>
       </c>
@@ -14874,7 +14870,7 @@
         <v>1609</v>
       </c>
     </row>
-    <row r="166" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="166" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A166" s="21" t="s">
         <v>407</v>
       </c>
@@ -14891,7 +14887,7 @@
         <v>1611</v>
       </c>
     </row>
-    <row r="167" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="167" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A167" s="21" t="s">
         <v>407</v>
       </c>
@@ -14908,7 +14904,7 @@
         <v>1613</v>
       </c>
     </row>
-    <row r="168" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="168" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A168" s="21" t="s">
         <v>407</v>
       </c>
@@ -14925,7 +14921,7 @@
         <v>1615</v>
       </c>
     </row>
-    <row r="169" spans="1:5" s="12" customFormat="1" ht="43.5">
+    <row r="169" spans="1:5" s="12" customFormat="1" ht="43.2">
       <c r="A169" s="21" t="s">
         <v>407</v>
       </c>
@@ -14942,7 +14938,7 @@
         <v>1617</v>
       </c>
     </row>
-    <row r="170" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="170" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A170" s="21" t="s">
         <v>407</v>
       </c>
@@ -14959,7 +14955,7 @@
         <v>1619</v>
       </c>
     </row>
-    <row r="171" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="171" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A171" s="21" t="s">
         <v>407</v>
       </c>
@@ -14976,7 +14972,7 @@
         <v>1621</v>
       </c>
     </row>
-    <row r="172" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="172" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A172" s="21" t="s">
         <v>407</v>
       </c>
@@ -14993,7 +14989,7 @@
         <v>1623</v>
       </c>
     </row>
-    <row r="173" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="173" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A173" s="21" t="s">
         <v>407</v>
       </c>
@@ -15010,7 +15006,7 @@
         <v>1625</v>
       </c>
     </row>
-    <row r="174" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="174" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A174" s="21" t="s">
         <v>407</v>
       </c>
@@ -15044,7 +15040,7 @@
         <v>1629</v>
       </c>
     </row>
-    <row r="176" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="176" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A176" s="21" t="s">
         <v>407</v>
       </c>
@@ -15061,7 +15057,7 @@
         <v>1631</v>
       </c>
     </row>
-    <row r="177" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="177" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A177" s="21" t="s">
         <v>407</v>
       </c>
@@ -15078,7 +15074,7 @@
         <v>1633</v>
       </c>
     </row>
-    <row r="178" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="178" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A178" s="21" t="s">
         <v>407</v>
       </c>
@@ -15095,7 +15091,7 @@
         <v>1635</v>
       </c>
     </row>
-    <row r="179" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="179" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A179" s="21" t="s">
         <v>407</v>
       </c>
@@ -15112,7 +15108,7 @@
         <v>1637</v>
       </c>
     </row>
-    <row r="180" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="180" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A180" s="21" t="s">
         <v>407</v>
       </c>
@@ -15129,7 +15125,7 @@
         <v>1639</v>
       </c>
     </row>
-    <row r="181" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="181" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A181" s="21" t="s">
         <v>407</v>
       </c>
@@ -15146,7 +15142,7 @@
         <v>1641</v>
       </c>
     </row>
-    <row r="182" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="182" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A182" s="21" t="s">
         <v>407</v>
       </c>
@@ -15163,7 +15159,7 @@
         <v>1643</v>
       </c>
     </row>
-    <row r="183" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="183" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A183" s="21" t="s">
         <v>407</v>
       </c>
@@ -15180,7 +15176,7 @@
         <v>1645</v>
       </c>
     </row>
-    <row r="184" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="184" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A184" s="21" t="s">
         <v>407</v>
       </c>
@@ -15197,7 +15193,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="185" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="185" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A185" s="21" t="s">
         <v>407</v>
       </c>
@@ -15214,7 +15210,7 @@
         <v>1649</v>
       </c>
     </row>
-    <row r="186" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="186" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A186" s="21" t="s">
         <v>407</v>
       </c>
@@ -15231,7 +15227,7 @@
         <v>1651</v>
       </c>
     </row>
-    <row r="187" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="187" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A187" s="21" t="s">
         <v>407</v>
       </c>
@@ -15265,7 +15261,7 @@
         <v>1655</v>
       </c>
     </row>
-    <row r="189" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="189" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A189" s="21" t="s">
         <v>407</v>
       </c>
@@ -15282,7 +15278,7 @@
         <v>1657</v>
       </c>
     </row>
-    <row r="190" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="190" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A190" s="21" t="s">
         <v>407</v>
       </c>
@@ -15316,7 +15312,7 @@
         <v>1661</v>
       </c>
     </row>
-    <row r="192" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="192" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A192" s="21" t="s">
         <v>407</v>
       </c>
@@ -15333,7 +15329,7 @@
         <v>1663</v>
       </c>
     </row>
-    <row r="193" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="193" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A193" s="21" t="s">
         <v>407</v>
       </c>
@@ -15350,7 +15346,7 @@
         <v>1665</v>
       </c>
     </row>
-    <row r="194" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="194" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A194" s="21" t="s">
         <v>407</v>
       </c>
@@ -15367,7 +15363,7 @@
         <v>1667</v>
       </c>
     </row>
-    <row r="195" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="195" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A195" s="21" t="s">
         <v>407</v>
       </c>
@@ -15384,7 +15380,7 @@
         <v>1669</v>
       </c>
     </row>
-    <row r="196" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="196" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A196" s="21" t="s">
         <v>407</v>
       </c>
@@ -15401,7 +15397,7 @@
         <v>1671</v>
       </c>
     </row>
-    <row r="197" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="197" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A197" s="21" t="s">
         <v>407</v>
       </c>
@@ -15418,7 +15414,7 @@
         <v>1673</v>
       </c>
     </row>
-    <row r="198" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="198" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A198" s="21" t="s">
         <v>407</v>
       </c>
@@ -15452,7 +15448,7 @@
         <v>1677</v>
       </c>
     </row>
-    <row r="200" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="200" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A200" s="21" t="s">
         <v>407</v>
       </c>
@@ -15486,7 +15482,7 @@
         <v>1681</v>
       </c>
     </row>
-    <row r="202" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="202" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A202" s="21" t="s">
         <v>407</v>
       </c>
@@ -15503,7 +15499,7 @@
         <v>1683</v>
       </c>
     </row>
-    <row r="203" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="203" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A203" s="21" t="s">
         <v>407</v>
       </c>
@@ -15520,7 +15516,7 @@
         <v>1685</v>
       </c>
     </row>
-    <row r="204" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="204" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A204" s="21" t="s">
         <v>407</v>
       </c>
@@ -15537,7 +15533,7 @@
         <v>1687</v>
       </c>
     </row>
-    <row r="205" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="205" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A205" s="21" t="s">
         <v>407</v>
       </c>
@@ -15554,7 +15550,7 @@
         <v>1689</v>
       </c>
     </row>
-    <row r="206" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="206" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A206" s="21" t="s">
         <v>407</v>
       </c>
@@ -15571,7 +15567,7 @@
         <v>1691</v>
       </c>
     </row>
-    <row r="207" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="207" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A207" s="21" t="s">
         <v>407</v>
       </c>
@@ -15588,7 +15584,7 @@
         <v>1693</v>
       </c>
     </row>
-    <row r="208" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="208" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A208" s="21" t="s">
         <v>407</v>
       </c>
@@ -15605,7 +15601,7 @@
         <v>1695</v>
       </c>
     </row>
-    <row r="209" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="209" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A209" s="21" t="s">
         <v>407</v>
       </c>
@@ -15622,7 +15618,7 @@
         <v>1697</v>
       </c>
     </row>
-    <row r="210" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="210" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A210" s="21" t="s">
         <v>407</v>
       </c>
@@ -15656,7 +15652,7 @@
         <v>1701</v>
       </c>
     </row>
-    <row r="212" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="212" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A212" s="21" t="s">
         <v>407</v>
       </c>
@@ -15673,7 +15669,7 @@
         <v>1703</v>
       </c>
     </row>
-    <row r="213" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="213" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A213" s="21" t="s">
         <v>407</v>
       </c>
@@ -15724,7 +15720,7 @@
         <v>1709</v>
       </c>
     </row>
-    <row r="216" spans="1:5" s="12" customFormat="1" ht="43.5">
+    <row r="216" spans="1:5" s="12" customFormat="1" ht="43.2">
       <c r="A216" s="21" t="s">
         <v>407</v>
       </c>
@@ -15741,7 +15737,7 @@
         <v>1711</v>
       </c>
     </row>
-    <row r="217" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="217" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A217" s="21" t="s">
         <v>407</v>
       </c>
@@ -15775,7 +15771,7 @@
         <v>1715</v>
       </c>
     </row>
-    <row r="219" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="219" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A219" s="21" t="s">
         <v>407</v>
       </c>
@@ -15792,7 +15788,7 @@
         <v>1717</v>
       </c>
     </row>
-    <row r="220" spans="1:5" s="12" customFormat="1" ht="29">
+    <row r="220" spans="1:5" s="12" customFormat="1" ht="28.8">
       <c r="A220" s="21" t="s">
         <v>407</v>
       </c>
@@ -16076,12 +16072,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8D30C07-B92F-494E-AD16-8F2C62A91261}">
   <dimension ref="A1:D56"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="25.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.81640625" customWidth="1"/>
-    <col min="4" max="4" width="26.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.77734375" customWidth="1"/>
+    <col min="4" max="4" width="26.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -16879,11 +16875,11 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{617E1E86-4318-4373-98CB-6362DB1DB101}">
   <dimension ref="A1:I764"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="5" max="5" width="27.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.88671875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -38334,9 +38330,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF0433E0-5026-4073-87CF-A04A4E545664}">
   <dimension ref="A1:A11"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="12.7265625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="12.77734375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">

</xml_diff>